<commit_message>
[AI]refactor: 对象池过期时间属性重命名 ExpireTime → ExpireTimeAfterIdle
- 语义修正：对象闲置（距上次使用或回收）超过该秒数即视为过期，纳入销毁候选
- ObjectPoolBase/ObjectPool 属性、字段、构造参数统一改名
- ExpireTime setter 由 DisposeOverCapacity 改为 DisposeExpired，设置后立即清理过期对象
- EntityGroup/UI 模块公开属性与配置表字段同步（PoolExpireTimeAfterIdle，去除 WinObj 前缀）
- 同步更新 Entity/UI/ObjectPool README 文档
</commit_message>
<xml_diff>
--- a/Config/Excels/Tables/E-EntityGroup-实体组配置表.xlsx
+++ b/Config/Excels/Tables/E-EntityGroup-实体组配置表.xlsx
@@ -23,13 +23,13 @@
     <t>Id</t>
   </si>
   <si>
-    <t>PoolAutoDisposeInterval</t>
+    <t>PoolAutoDisposeCheckInterval</t>
   </si>
   <si>
     <t>PoolCapacity</t>
   </si>
   <si>
-    <t>PoolExpireTime</t>
+    <t>PoolExpireTimeAfterIdle</t>
   </si>
   <si>
     <t>PoolPriority</t>
@@ -56,16 +56,16 @@
     <t>实体组ID</t>
   </si>
   <si>
-    <t>自动释放间隔(秒)</t>
-  </si>
-  <si>
-    <t>对象池容量</t>
-  </si>
-  <si>
-    <t>对象过期时间(秒)</t>
-  </si>
-  <si>
-    <t>对象池优先级</t>
+    <t>实体对象池自动销毁检查间隔(秒)</t>
+  </si>
+  <si>
+    <t>实体对象池容量</t>
+  </si>
+  <si>
+    <t>实体对象闲置后过期秒数</t>
+  </si>
+  <si>
+    <t>实体对象池优先级</t>
   </si>
   <si>
     <t>Player</t>
@@ -116,9 +116,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -140,13 +139,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -154,7 +146,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -169,7 +169,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -199,6 +207,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="宋体"/>
@@ -206,40 +222,24 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -247,7 +247,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -268,181 +268,181 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -471,17 +471,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -489,8 +483,23 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -506,6 +515,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -530,21 +554,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -559,25 +568,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -586,133 +586,133 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1081,9 +1081,9 @@
   <cols>
     <col min="1" max="1" width="9" style="1"/>
     <col min="2" max="2" width="18.375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="29.375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="38.125" style="2" customWidth="1"/>
     <col min="4" max="4" width="17.75" style="2" customWidth="1"/>
-    <col min="5" max="5" width="20.875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="29.75" style="2" customWidth="1"/>
     <col min="6" max="6" width="18" style="2" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>